<commit_message>
treating files differently especially in main.py
</commit_message>
<xml_diff>
--- a/data/ExcelParameters/CapacityPerChannel.xlsx
+++ b/data/ExcelParameters/CapacityPerChannel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://loreal-my.sharepoint.com/personal/nils_levillain_loreal_com/Documents/Desktop/Python/WindSurf/Test/ExcelParameters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://loreal-my.sharepoint.com/personal/nils_levillain_loreal_com/Documents/Documents/Cline/nw-allocation-tool/data/ExcelParameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC890B24-8725-43BD-BBB8-D8DEF3A8916D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{BC890B24-8725-43BD-BBB8-D8DEF3A8916D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E6BBDA8-142C-469F-B2F2-91CE25570F39}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CA5851D4-C131-4FE7-9ED9-D1418C4549E6}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{CA5851D4-C131-4FE7-9ED9-D1418C4549E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -38,18 +38,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="16">
   <si>
-    <t>Channel</t>
-  </si>
-  <si>
     <t>operational_division</t>
   </si>
   <si>
     <t>operational_axe_label</t>
   </si>
   <si>
-    <t>Max capacity (in # of SKU)</t>
-  </si>
-  <si>
     <t>Outlet</t>
   </si>
   <si>
@@ -84,6 +78,12 @@
   </si>
   <si>
     <t>PPD</t>
+  </si>
+  <si>
+    <t>max_skus</t>
+  </si>
+  <si>
+    <t>channel_id</t>
   </si>
 </sst>
 </file>
@@ -326,23 +326,23 @@
       </border>
     </dxf>
     <dxf>
-      <border>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
+      <border>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -380,13 +380,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BBA06785-E0A1-4589-9DE3-7AB38C93DFB7}" name="Tableau6" displayName="Tableau6" ref="A1:D29" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BBA06785-E0A1-4589-9DE3-7AB38C93DFB7}" name="Tableau6" displayName="Tableau6" ref="A1:D29" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A1:D29" xr:uid="{BBA06785-E0A1-4589-9DE3-7AB38C93DFB7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{5DA93ED5-04E6-40EE-9CFC-5078C38FBABA}" name="Channel" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{5DA93ED5-04E6-40EE-9CFC-5078C38FBABA}" name="channel_id" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{BC74846B-F88C-40AC-A0A0-B7A60BC635CE}" name="operational_division" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{13CD1147-CC13-4CB2-9C7F-A4D7415E8779}" name="operational_axe_label" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{A6CA7BC0-E659-492E-8F8C-112D1B7C574E}" name="Max capacity (in # of SKU)" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{A6CA7BC0-E659-492E-8F8C-112D1B7C574E}" name="max_skus" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -712,7 +712,7 @@
   <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.1796875" bestFit="1" customWidth="1"/>
@@ -720,27 +720,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>6</v>
       </c>
       <c r="D2" s="6">
         <v>300</v>
@@ -748,13 +748,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>5</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>7</v>
       </c>
       <c r="D3" s="6">
         <v>100</v>
@@ -762,13 +762,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D4" s="6">
         <v>3500</v>
@@ -776,13 +776,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" s="6">
         <v>1500</v>
@@ -790,13 +790,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D6" s="6">
         <v>65000</v>
@@ -804,13 +804,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D7" s="6">
         <v>500</v>
@@ -818,13 +818,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D8" s="6">
         <v>6000</v>
@@ -832,13 +832,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>6</v>
       </c>
       <c r="D9" s="6">
         <v>0</v>
@@ -846,13 +846,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="6">
         <v>0</v>
@@ -860,13 +860,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D11" s="6">
         <v>0</v>
@@ -874,13 +874,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D12" s="6">
         <v>0</v>
@@ -888,13 +888,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D13" s="6">
         <v>0</v>
@@ -902,13 +902,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D14" s="6">
         <v>0</v>
@@ -916,13 +916,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D15" s="6">
         <v>1500</v>
@@ -930,13 +930,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>6</v>
       </c>
       <c r="D16" s="6">
         <v>5000</v>
@@ -944,13 +944,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D17" s="6">
         <v>0</v>
@@ -958,13 +958,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D18" s="6">
         <v>0</v>
@@ -972,13 +972,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D19" s="6">
         <v>0</v>
@@ -986,13 +986,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D20" s="6">
         <v>15000</v>
@@ -1000,13 +1000,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D21" s="6">
         <v>0</v>
@@ -1014,13 +1014,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D22" s="6">
         <v>3000</v>
@@ -1028,13 +1028,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>6</v>
       </c>
       <c r="D23" s="6">
         <v>0</v>
@@ -1042,13 +1042,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D24" s="6">
         <v>0</v>
@@ -1056,13 +1056,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D25" s="6">
         <v>1500</v>
@@ -1070,13 +1070,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D26" s="6">
         <v>0</v>
@@ -1084,13 +1084,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D27" s="6">
         <v>0</v>
@@ -1098,13 +1098,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D28" s="6">
         <v>0</v>
@@ -1112,13 +1112,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D29" s="6">
         <v>0</v>

</xml_diff>